<commit_message>
Fix false negative logic in risk engine and normalize Quote Guard
</commit_message>
<xml_diff>
--- a/data/Meridian_Vendor_Output.xlsx
+++ b/data/Meridian_Vendor_Output.xlsx
@@ -1039,7 +1039,7 @@
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] No</t>
+          <t>[MOCK] Inconclusive</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] N/A — no public evidence of AI usage in the service provided to Meridian.</t>
+          <t>[MOCK] Weak or marketing-level signals detected. Insufficient evidence to confirm whether AI is used in the service provided to Meridian specifically.</t>
         </is>
       </c>
       <c r="R6" s="3" t="inlineStr">
@@ -1061,17 +1061,17 @@
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] None identified</t>
+          <t>[MOCK] Medium</t>
         </is>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>No public evidence of AI usage. 6 coverage gap(s) recorded. Rating subject to the caveat that absence of evidence is not evidence of absence.</t>
+          <t>Vendor has Low criticality tier. Insufficient coverage (1 pages checked, 6 gaps) to confirm absence of AI. Provisional rating applied.</t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
         <is>
-          <t>Monitor annually. No immediate action required based on current public evidence.</t>
+          <t>Issue an AI usage questionnaire to clarify whether AI is used in the service provided to Meridian. Include questions on model providers, data handling, and oversight. Flag for follow-up review in next assessment cycle.</t>
         </is>
       </c>
       <c r="V6" s="3" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>No public evidence of AI usage. 14 coverage gap(s) recorded. Rating subject to the caveat that absence of evidence is not evidence of absence.</t>
+          <t>No public evidence of AI usage across adequate coverage (3 pages checked). Rating subject to the caveat that absence of evidence is not evidence of absence.</t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>No public evidence of AI usage. 10 coverage gap(s) recorded. Rating subject to the caveat that absence of evidence is not evidence of absence.</t>
+          <t>No public evidence of AI usage across adequate coverage (3 pages checked). Rating subject to the caveat that absence of evidence is not evidence of absence.</t>
         </is>
       </c>
       <c r="U8" s="3" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] No</t>
+          <t>[MOCK] Inconclusive</t>
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] N/A — no public evidence of AI usage in the service provided to Meridian.</t>
+          <t>[MOCK] Weak or marketing-level signals detected. Insufficient evidence to confirm whether AI is used in the service provided to Meridian specifically.</t>
         </is>
       </c>
       <c r="R9" s="3" t="inlineStr">
@@ -1388,17 +1388,17 @@
       </c>
       <c r="S9" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] None identified</t>
+          <t>[MOCK] Medium</t>
         </is>
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>No public evidence of AI usage. 8 coverage gap(s) recorded. Rating subject to the caveat that absence of evidence is not evidence of absence.</t>
+          <t>Vendor has Medium criticality tier. Insufficient coverage (0 pages checked, 8 gaps) to confirm absence of AI. Provisional rating applied.</t>
         </is>
       </c>
       <c r="U9" s="3" t="inlineStr">
         <is>
-          <t>Monitor annually. No immediate action required based on current public evidence.</t>
+          <t>Issue an AI usage questionnaire to clarify whether AI is used in the service provided to Meridian. Include questions on model providers, data handling, and oversight. Flag for follow-up review in next assessment cycle.</t>
         </is>
       </c>
       <c r="V9" s="3" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="T11" s="3" t="inlineStr">
         <is>
-          <t>No public evidence of AI usage. 0 coverage gap(s) recorded. Rating subject to the caveat that absence of evidence is not evidence of absence.</t>
+          <t>No public evidence of AI usage across adequate coverage (17 pages checked). Rating subject to the caveat that absence of evidence is not evidence of absence.</t>
         </is>
       </c>
       <c r="U11" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Apply Sonnet's M2 collector v2 rewrite and risk engine logic fixes
</commit_message>
<xml_diff>
--- a/data/Meridian_Vendor_Output.xlsx
+++ b/data/Meridian_Vendor_Output.xlsx
@@ -1039,19 +1039,19 @@
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] Inconclusive</t>
+          <t>No</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
           <t>No indicative AI evidence found.
-Sources successfully checked (1): https://www.automworx.com
+Sources successfully checked (3): https://www.automworx.com, https://www.automworx.com/privacy-policy, https://www.automworx.com/webinar-using-the-automic-rest-api-to-integrate-with-servicenow
 Coverage gaps (6): https://www.automworx.com/ai-policy, https://www.automworx.com/docs, https://www.automworx.com/dpa, https://www.automworx.com/security, https://www.automworx.com/subprocessors</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] Weak or marketing-level signals detected. Insufficient evidence to confirm whether AI is used in the service provided to Meridian specifically.</t>
+          <t>N/A — no public evidence of AI usage in the service provided to Meridian.</t>
         </is>
       </c>
       <c r="R6" s="3" t="inlineStr">
@@ -1061,17 +1061,17 @@
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] Medium</t>
+          <t>None identified</t>
         </is>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>Vendor has Low criticality tier. Insufficient coverage (1 pages checked, 6 gaps) to confirm absence of AI. Provisional rating applied.</t>
+          <t>No public evidence of AI usage across adequate coverage (3 pages checked). Rating subject to the caveat that absence of evidence is not evidence of absence.</t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
         <is>
-          <t>Issue an AI usage questionnaire to clarify whether AI is used in the service provided to Meridian. Include questions on model providers, data handling, and oversight. Flag for follow-up review in next assessment cycle.</t>
+          <t>Monitor annually. No immediate action required based on current public evidence.</t>
         </is>
       </c>
       <c r="V6" s="3" t="inlineStr">
@@ -1148,39 +1148,51 @@
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] No</t>
+          <t>Inconclusive</t>
         </is>
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>No indicative AI evidence found.
-Sources successfully checked (3): https://www.fiserv.com, https://www.fiserv.com/, https://www.fiserv.com/careers
-Coverage gaps (14): https://www.fiserv.com/about, https://www.fiserv.com/ai-policy, https://www.fiserv.com/api, https://www.fiserv.com/blog, https://www.fiserv.com/developers</t>
+          <t>"|  | Advanced detection techniques Leverage AI-driven risk scoring to analyze transaction patterns and customer behavior in real time."
+Source: https://www.fiserv.com/en/solutions/risk-compliance/aml-risk-manager.html (retrieved 2026-10-10)
+"Our approach includes:
+- Ongoing investment in cybersecurity and technology modernization
+- Continuous monitoring and proactive risk management
+- Security-focused software development and deployment practices
+- Collaboration with industry partners and security initiatives
+- Resilience testing and operational preparedness
+- Continuous enhancement of defensive capabilities to address emerging AI-enabled threats
+As the threat landscape continues to evolve, Fiserv remains committed to helping clients operate securely through defined cybersecurity practices, reliable technology platforms, and ongoing innovation."
+Source: https://www.fiserv.com/en/legal/cybersecurity.html (retrieved 2026-10-10)
+"Cybersecurity Best Practices in a Rapidly Evolving Threat Environment
+Security and Resilience in the Age of AI
+The cybersecurity landscape is evolving rapidly as bad actors increasingly use artificial intelligence to identify, automate, and exploit technology vulnerabilities at greater speed and scale."
+Source: https://www.fiserv.com/en/legal/cybersecurity.html (retrieved 2026-10-10)</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] N/A — no public evidence of AI usage in the service provided to Meridian.</t>
+          <t>Weak or marketing-level signals detected. Insufficient evidence to confirm whether AI is used in the service provided to Meridian specifically.</t>
         </is>
       </c>
       <c r="R7" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>None named — Inconclusive. No sub-processor register or AI policy found publicly.</t>
         </is>
       </c>
       <c r="S7" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] None identified</t>
+          <t>High</t>
         </is>
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>No public evidence of AI usage across adequate coverage (3 pages checked). Rating subject to the caveat that absence of evidence is not evidence of absence.</t>
+          <t>Vendor has Critical criticality tier. Weak AI signals detected (score: 8.4) but insufficient to confirm service-specific usage. Provisional rating based on criticality and data class ("Full customer master, balances and transactions for 1.4 million customers.").</t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr">
         <is>
-          <t>Monitor annually. No immediate action required based on current public evidence.</t>
+          <t>Issue an AI usage questionnaire to clarify whether AI is used in the service provided to Meridian. Include questions on model providers, data handling, and oversight. Flag for follow-up review in next assessment cycle.</t>
         </is>
       </c>
       <c r="V7" s="3" t="inlineStr">
@@ -1257,19 +1269,19 @@
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] No</t>
+          <t>No</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
           <t>No indicative AI evidence found.
-Sources successfully checked (3): https://www.fssi-ca.com, https://www.fssi-ca.com/blog, https://www.fssi-ca.com/jobs
-Coverage gaps (10): https://www.fssi-ca.com/ai-policy, https://www.fssi-ca.com/api, https://www.fssi-ca.com/careers, https://www.fssi-ca.com/developers, https://www.fssi-ca.com/docs</t>
+Sources successfully checked (13): https://www.fssi-ca.com, https://www.fssi-ca.com/capabilities/regulatory-compliance, https://www.fssi-ca.com/cybersecurity-awareness-month-2021-data-security-tips, https://www.fssi-ca.com/improving-the-data-security-and-privacy-of-your-organization, https://www.fssi-ca.com/infrastructure/hipaa-compliance, https://www.fssi-ca.com/optimizing-transactional-document-delivery-for-the-alarm-and-security-industry, https://www.fssi-ca.com/print-and-mail-compliance-guide-for-secure-document-processing, https://www.fssi-ca.com/privacy
+Coverage gaps (11): https://www.fssi-ca.com/ai-policy, https://www.fssi-ca.com/docs, https://www.fssi-ca.com/dpa, https://www.fssi-ca.com/security, https://www.fssi-ca.com/subprocessors</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] N/A — no public evidence of AI usage in the service provided to Meridian.</t>
+          <t>N/A — no public evidence of AI usage in the service provided to Meridian.</t>
         </is>
       </c>
       <c r="R8" s="3" t="inlineStr">
@@ -1279,12 +1291,12 @@
       </c>
       <c r="S8" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] None identified</t>
+          <t>None identified</t>
         </is>
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>No public evidence of AI usage across adequate coverage (3 pages checked). Rating subject to the caveat that absence of evidence is not evidence of absence.</t>
+          <t>No public evidence of AI usage across adequate coverage (13 pages checked). Rating subject to the caveat that absence of evidence is not evidence of absence.</t>
         </is>
       </c>
       <c r="U8" s="3" t="inlineStr">
@@ -1366,34 +1378,34 @@
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] Inconclusive</t>
+          <t>Inconclusive</t>
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
           <t>No indicative AI evidence found.
 Sources successfully checked (0): 
-Coverage gaps (8): https://www.terrapintech.com, https://www.terrapintech.com/, https://www.terrapintech.com/api, https://www.terrapintech.com/blog, https://www.terrapintech.com/careers</t>
+Coverage gaps (7): https://www.terrapintech.com, https://www.terrapintech.com/api, https://www.terrapintech.com/blog, https://www.terrapintech.com/careers, https://www.terrapintech.com/developers</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] Weak or marketing-level signals detected. Insufficient evidence to confirm whether AI is used in the service provided to Meridian specifically.</t>
+          <t>Insufficient coverage; no determination possible.</t>
         </is>
       </c>
       <c r="R9" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>None named — Inconclusive. No sub-processor register or AI policy found publicly.</t>
         </is>
       </c>
       <c r="S9" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] Medium</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>Vendor has Medium criticality tier. Insufficient coverage (0 pages checked, 8 gaps) to confirm absence of AI. Provisional rating applied.</t>
+          <t>Vendor has Medium criticality tier. Insufficient coverage (0 pages checked, 7 gaps) to confirm absence of AI. Provisional rating applied.</t>
         </is>
       </c>
       <c r="U9" s="3" t="inlineStr">
@@ -1475,7 +1487,7 @@
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] Inconclusive</t>
+          <t>Inconclusive</t>
         </is>
       </c>
       <c r="P10" s="3" t="inlineStr">
@@ -1485,30 +1497,27 @@
   - “Artificial Intelligence” means any technology that enables machines to perform tasks that typically require human intelligence, including but not limited to generative AI, machine learning, natural language processing, and computer vision."
 Source: https://www.bny.com/ai-policy (retrieved 2026-10-10)
 "This Acceptable Use Policy (“Policy”) applies to Your use of all services offered by BNY or third-party products, applications, or functionality that interoperate with services offered by BNY, that incorporate Artificial Intelligence, including proprietary and third-party solutions (each, an “AI Service”)."
-Source: https://www.bny.com/ai-policy (retrieved 2026-10-10)
-"DATA &amp; ANALYTICS
-Cloud-native and AI enabled platform for data and operations."
-Source: https://www.bny.com (retrieved 2026-10-10)</t>
+Source: https://www.bny.com/ai-policy (retrieved 2026-10-10)</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] Weak or marketing-level signals detected. Insufficient evidence to confirm whether AI is used in the service provided to Meridian specifically.</t>
+          <t>Weak or marketing-level signals detected. Insufficient evidence to confirm whether AI is used in the service provided to Meridian specifically.</t>
         </is>
       </c>
       <c r="R10" s="3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>None named — Inconclusive. No sub-processor register or AI policy found publicly.</t>
         </is>
       </c>
       <c r="S10" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] High</t>
+          <t>High</t>
         </is>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>Vendor has High criticality tier. Weak AI signals detected (score: 3.5) but insufficient to confirm service-specific usage. Provisional rating based on criticality and data class ("Payment instructions, counterparty names and account identifiers.").</t>
+          <t>Vendor has High criticality tier. Weak AI signals detected (score: 3.3) but insufficient to confirm service-specific usage. Provisional rating based on criticality and data class ("Payment instructions, counterparty names and account identifiers.").</t>
         </is>
       </c>
       <c r="U10" s="3" t="inlineStr">
@@ -1590,18 +1599,19 @@
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] No</t>
+          <t>No</t>
         </is>
       </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
           <t>No indicative AI evidence found.
-Sources successfully checked (17): https://www.theclearinghouse.org, https://www.theclearinghouse.org/, https://www.theclearinghouse.org/about, https://www.theclearinghouse.org/ai-policy, https://www.theclearinghouse.org/api, https://www.theclearinghouse.org/blog, https://www.theclearinghouse.org/careers, https://www.theclearinghouse.org/developers</t>
+Sources successfully checked (18): https://www.theclearinghouse.org, https://www.theclearinghouse.org/forms-old/rtp-compliance-implications, https://www.theclearinghouse.org/forms-old/rtp-network-rules-compliance-enforcement, https://www.theclearinghouse.org/payment-systems/articles/2018/08/data-privacy-08-21-2018, https://www.theclearinghouse.org/payment-systems/articles/2018/10/data-privacy-10-18-2018, https://www.theclearinghouse.org/payment-systems/articles/2019/07/071119-heritage-trust, https://www.theclearinghouse.org/payment-systems/articles/2024/07/cfpb-compliance-deadline, https://www.theclearinghouse.org/payment-systems/rtp/technical-documentation
+Coverage gaps (18): https://www.theclearinghouse.org/ai-policy, https://www.theclearinghouse.org/docs, https://www.theclearinghouse.org/dpa, https://www.theclearinghouse.org/payments-services/education/ach/compliance-risk-management, https://www.theclearinghouse.org/payments-services/education/corporate/compliance-risk-management</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] N/A — no public evidence of AI usage in the service provided to Meridian.</t>
+          <t>N/A — no public evidence of AI usage in the service provided to Meridian.</t>
         </is>
       </c>
       <c r="R11" s="3" t="inlineStr">
@@ -1611,12 +1621,12 @@
       </c>
       <c r="S11" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] None identified</t>
+          <t>None identified</t>
         </is>
       </c>
       <c r="T11" s="3" t="inlineStr">
         <is>
-          <t>No public evidence of AI usage across adequate coverage (17 pages checked). Rating subject to the caveat that absence of evidence is not evidence of absence.</t>
+          <t>No public evidence of AI usage across adequate coverage (18 pages checked). Rating subject to the caveat that absence of evidence is not evidence of absence.</t>
         </is>
       </c>
       <c r="U11" s="3" t="inlineStr">
@@ -2149,7 +2159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2197,129 +2207,221 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>V-002</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.fiserv.com/en/solutions/risk-compliance/aml-risk-manager.html</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Tier_A</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://www.fiserv.com/en/solutions/risk-compliance/aml-risk-manager.html</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-10-10T06:17:40.484938+00:00</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>|  | Advanced detection techniques Leverage AI-driven risk scoring to analyze transaction patterns and customer behavior in real time.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>INDICATIVE</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>bbf9f86093b9ffb25ab6aed003eaf13162c0712252e6bdfdd50cf8312e0dbda0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>V-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.fiserv.com/en/legal/cybersecurity.html</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Tier_A</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.fiserv.com/en/legal/cybersecurity.html</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-10-10T06:17:27.063871+00:00</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Our approach includes:
+- Ongoing investment in cybersecurity and technology modernization
+- Continuous monitoring and proactive risk management
+- Security-focused software development and deployment practices
+- Collaboration with industry partners and security initiatives
+- Resilience testing and operational preparedness
+- Continuous enhancement of defensive capabilities to address emerging AI-enabled threats
+As the threat landscape continues to evolve, Fiserv remains committed to helping clients operate securely through defined cybersecurity practices, reliable technology platforms, and ongoing innovation.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>MARKETING-ONLY</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>c8ae42b7ee474576c84822b5f8d2a9e306f7e26ed7e7a10c1198ff5990595d35</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>V-002</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.fiserv.com/en/legal/cybersecurity.html</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Tier_A</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.fiserv.com/en/legal/cybersecurity.html</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-10-10T06:17:27.063871+00:00</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Cybersecurity Best Practices in a Rapidly Evolving Threat Environment
+Security and Resilience in the Age of AI
+The cybersecurity landscape is evolving rapidly as bad actors increasingly use artificial intelligence to identify, automate, and exploit technology vulnerabilities at greater speed and scale.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>MARKETING-ONLY</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>c8ae42b7ee474576c84822b5f8d2a9e306f7e26ed7e7a10c1198ff5990595d35</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>V-005</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>https://www.bny.com/ai-policy</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Tier_A</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>https://www.bny.com/ai-policy</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-10-10T04:42:56.353288+00:00</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-10-10T06:19:45.726343+00:00</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>- Definitions
  For the purposes of this Policy:
   - “Artificial Intelligence” means any technology that enables machines to perform tasks that typically require human intelligence, including but not limited to generative AI, machine learning, natural language processing, and computer vision.</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>INDICATIVE</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>b31b1f0ef72c6f75f441627dd1e3e12b5305831bc8980275fa4a514304f1d512</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>V-005</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>https://www.bny.com/ai-policy</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Tier_A</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>https://www.bny.com/ai-policy</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-10-10T04:42:56.353288+00:00</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-10-10T06:19:45.726343+00:00</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>This Acceptable Use Policy (“Policy”) applies to Your use of all services offered by BNY or third-party products, applications, or functionality that interoperate with services offered by BNY, that incorporate Artificial Intelligence, including proprietary and third-party solutions (each, an “AI Service”).</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>MARKETING-ONLY</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>b31b1f0ef72c6f75f441627dd1e3e12b5305831bc8980275fa4a514304f1d512</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>V-005</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://www.bny.com</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Tier_D</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.bny.com</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-10-10T04:42:54.169759+00:00</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>DATA &amp; ANALYTICS
-Cloud-native and AI enabled platform for data and operations.</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>MARKETING-ONLY</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>848ffca667031a7927323e7f82ea67d2e2d1800c19824f5d5032e57536d4de82</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix silent mock fallback preventing [MOCK] watermark
</commit_message>
<xml_diff>
--- a/data/Meridian_Vendor_Output.xlsx
+++ b/data/Meridian_Vendor_Output.xlsx
@@ -1039,7 +1039,7 @@
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>[MOCK] No</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>N/A — no public evidence of AI usage in the service provided to Meridian.</t>
+          <t>[MOCK] N/A — no public evidence of AI usage in the service provided to Meridian.</t>
         </is>
       </c>
       <c r="R6" s="3" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>None identified</t>
+          <t>[MOCK] None identified</t>
         </is>
       </c>
       <c r="T6" s="3" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>Inconclusive</t>
+          <t>[MOCK] Inconclusive</t>
         </is>
       </c>
       <c r="P7" s="3" t="inlineStr">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>Weak or marketing-level signals detected. Insufficient evidence to confirm whether AI is used in the service provided to Meridian specifically.</t>
+          <t>[MOCK] Weak or marketing-level signals detected. Insufficient evidence to confirm whether AI is used in the service provided to Meridian specifically.</t>
         </is>
       </c>
       <c r="R7" s="3" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="S7" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>[MOCK] High</t>
         </is>
       </c>
       <c r="T7" s="3" t="inlineStr">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>[MOCK] No</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>N/A — no public evidence of AI usage in the service provided to Meridian.</t>
+          <t>[MOCK] N/A — no public evidence of AI usage in the service provided to Meridian.</t>
         </is>
       </c>
       <c r="R8" s="3" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="S8" s="3" t="inlineStr">
         <is>
-          <t>None identified</t>
+          <t>[MOCK] None identified</t>
         </is>
       </c>
       <c r="T8" s="3" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>Inconclusive</t>
+          <t>[MOCK] Inconclusive</t>
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>Insufficient coverage; no determination possible.</t>
+          <t>[MOCK] Insufficient coverage; no determination possible.</t>
         </is>
       </c>
       <c r="R9" s="3" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="S9" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>[MOCK] Medium</t>
         </is>
       </c>
       <c r="T9" s="3" t="inlineStr">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>Inconclusive</t>
+          <t>[MOCK] Inconclusive</t>
         </is>
       </c>
       <c r="P10" s="3" t="inlineStr">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>Weak or marketing-level signals detected. Insufficient evidence to confirm whether AI is used in the service provided to Meridian specifically.</t>
+          <t>[MOCK] Weak or marketing-level signals detected. Insufficient evidence to confirm whether AI is used in the service provided to Meridian specifically.</t>
         </is>
       </c>
       <c r="R10" s="3" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="S10" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>[MOCK] High</t>
         </is>
       </c>
       <c r="T10" s="3" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>[MOCK] No</t>
         </is>
       </c>
       <c r="P11" s="3" t="inlineStr">
@@ -1611,7 +1611,7 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>N/A — no public evidence of AI usage in the service provided to Meridian.</t>
+          <t>[MOCK] N/A — no public evidence of AI usage in the service provided to Meridian.</t>
         </is>
       </c>
       <c r="R11" s="3" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="S11" s="3" t="inlineStr">
         <is>
-          <t>None identified</t>
+          <t>[MOCK] None identified</t>
         </is>
       </c>
       <c r="T11" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add native local Ollama support for free LLM inference
</commit_message>
<xml_diff>
--- a/data/Meridian_Vendor_Output.xlsx
+++ b/data/Meridian_Vendor_Output.xlsx
@@ -1039,7 +1039,7 @@
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] No</t>
+          <t>No</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] N/A — no public evidence of AI usage in the service provided to Meridian.</t>
+          <t>N/A — no public evidence of AI usage in the service provided to Meridian.</t>
         </is>
       </c>
       <c r="R6" s="3" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] None identified</t>
+          <t>None identified</t>
         </is>
       </c>
       <c r="T6" s="3" t="inlineStr">
@@ -1148,31 +1148,20 @@
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] Inconclusive</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>"|  | Advanced detection techniques Leverage AI-driven risk scoring to analyze transaction patterns and customer behavior in real time."
+          <t>"Leverage AI-driven risk scoring to analyze transaction patterns and customer behavior in real time."
 Source: https://www.fiserv.com/en/solutions/risk-compliance/aml-risk-manager.html (retrieved 2026-10-10)
-"Our approach includes:
-- Ongoing investment in cybersecurity and technology modernization
-- Continuous monitoring and proactive risk management
-- Security-focused software development and deployment practices
-- Collaboration with industry partners and security initiatives
-- Resilience testing and operational preparedness
-- Continuous enhancement of defensive capabilities to address emerging AI-enabled threats
-As the threat landscape continues to evolve, Fiserv remains committed to helping clients operate securely through defined cybersecurity practices, reliable technology platforms, and ongoing innovation."
-Source: https://www.fiserv.com/en/legal/cybersecurity.html (retrieved 2026-10-10)
-"Cybersecurity Best Practices in a Rapidly Evolving Threat Environment
-Security and Resilience in the Age of AI
-The cybersecurity landscape is evolving rapidly as bad actors increasingly use artificial intelligence to identify, automate, and exploit technology vulnerabilities at greater speed and scale."
+"The cybersecurity landscape is evolving rapidly as bad actors increasingly use artificial intelligence to identify, automate, and exploit technology vulnerabilities at greater speed and scale."
 Source: https://www.fiserv.com/en/legal/cybersecurity.html (retrieved 2026-10-10)</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] Weak or marketing-level signals detected. Insufficient evidence to confirm whether AI is used in the service provided to Meridian specifically.</t>
+          <t>risk scoring; Identifying, automating, and exploiting technology vulnerabilities</t>
         </is>
       </c>
       <c r="R7" s="3" t="inlineStr">
@@ -1182,17 +1171,17 @@
       </c>
       <c r="S7" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>Vendor has Critical criticality tier. Weak AI signals detected (score: 8.4) but insufficient to confirm service-specific usage. Provisional rating based on criticality and data class ("Full customer master, balances and transactions for 1.4 million customers.").</t>
+          <t>Vendor has Critical criticality tier with confirmed AI footprint. Data accessed includes "Full customer master, balances and transactions for 1.4 million customers.". Weighted evidence score: 32.4 across 2 valid signal(s). No model provider is publicly identified, leaving data flows untraceable. Evidence strength: strong.</t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr">
         <is>
-          <t>Issue an AI usage questionnaire to clarify whether AI is used in the service provided to Meridian. Include questions on model providers, data handling, and oversight. Flag for follow-up review in next assessment cycle.</t>
+          <t>Issue a targeted AI questionnaire within 15 business days covering: (1) model provider identity, hosting region, and data retention policy; (2) whether Meridian data (Full customer master, balances and transactions for 1.4 million customers.) is processed by AI models; (3) human review controls over AI-generated outputs. Register the vendor on the AI sub-processor inventory with an unresolved-provider flag. Raise AI-specific contract clauses at next review, addressing training restrictions, sub-processor change notification, and rights to audit. Escalate to Third-Party Risk Committee if confirmation not received within 30 days.</t>
         </is>
       </c>
       <c r="V7" s="3" t="inlineStr">
@@ -1269,7 +1258,7 @@
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] No</t>
+          <t>No</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
@@ -1281,7 +1270,7 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] N/A — no public evidence of AI usage in the service provided to Meridian.</t>
+          <t>N/A — no public evidence of AI usage in the service provided to Meridian.</t>
         </is>
       </c>
       <c r="R8" s="3" t="inlineStr">
@@ -1291,7 +1280,7 @@
       </c>
       <c r="S8" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] None identified</t>
+          <t>None identified</t>
         </is>
       </c>
       <c r="T8" s="3" t="inlineStr">
@@ -1378,7 +1367,7 @@
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] Inconclusive</t>
+          <t>Inconclusive</t>
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr">
@@ -1390,7 +1379,7 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] Insufficient coverage; no determination possible.</t>
+          <t>Insufficient coverage; no determination possible.</t>
         </is>
       </c>
       <c r="R9" s="3" t="inlineStr">
@@ -1400,7 +1389,7 @@
       </c>
       <c r="S9" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] Medium</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="T9" s="3" t="inlineStr">
@@ -1487,22 +1476,18 @@
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] Inconclusive</t>
+          <t>Inconclusive</t>
         </is>
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
-          <t>"- Definitions
- For the purposes of this Policy:
-  - “Artificial Intelligence” means any technology that enables machines to perform tasks that typically require human intelligence, including but not limited to generative AI, machine learning, natural language processing, and computer vision."
-Source: https://www.bny.com/ai-policy (retrieved 2026-10-10)
-"This Acceptable Use Policy (“Policy”) applies to Your use of all services offered by BNY or third-party products, applications, or functionality that interoperate with services offered by BNY, that incorporate Artificial Intelligence, including proprietary and third-party solutions (each, an “AI Service”)."
+          <t>"Use any robot, spider, intelligent agent, other automatic device or manual process, or automated systems to search, monitor or copy our web pages, data, content or other materials contained herein"
 Source: https://www.bny.com/ai-policy (retrieved 2026-10-10)</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] Weak or marketing-level signals detected. Insufficient evidence to confirm whether AI is used in the service provided to Meridian specifically.</t>
+          <t>Weak or marketing-level signals detected. Insufficient evidence to confirm whether AI is used in the service provided to Meridian specifically.</t>
         </is>
       </c>
       <c r="R10" s="3" t="inlineStr">
@@ -1512,12 +1497,12 @@
       </c>
       <c r="S10" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] High</t>
+          <t>High</t>
         </is>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>Vendor has High criticality tier. Weak AI signals detected (score: 3.3) but insufficient to confirm service-specific usage. Provisional rating based on criticality and data class ("Payment instructions, counterparty names and account identifiers.").</t>
+          <t>Vendor has High criticality tier. Weak AI signals detected (score: 0.9) but insufficient to confirm service-specific usage. Provisional rating based on criticality and data class ("Payment instructions, counterparty names and account identifiers.").</t>
         </is>
       </c>
       <c r="U10" s="3" t="inlineStr">
@@ -1599,7 +1584,7 @@
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] No</t>
+          <t>No</t>
         </is>
       </c>
       <c r="P11" s="3" t="inlineStr">
@@ -1611,7 +1596,7 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] N/A — no public evidence of AI usage in the service provided to Meridian.</t>
+          <t>N/A — no public evidence of AI usage in the service provided to Meridian.</t>
         </is>
       </c>
       <c r="R11" s="3" t="inlineStr">
@@ -1621,7 +1606,7 @@
       </c>
       <c r="S11" s="3" t="inlineStr">
         <is>
-          <t>[MOCK] None identified</t>
+          <t>None identified</t>
         </is>
       </c>
       <c r="T11" s="3" t="inlineStr">
@@ -2159,7 +2144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2232,12 +2217,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>|  | Advanced detection techniques Leverage AI-driven risk scoring to analyze transaction patterns and customer behavior in real time.</t>
+          <t>Leverage AI-driven risk scoring to analyze transaction patterns and customer behavior in real time.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>INDICATIVE</t>
+          <t>CONFIRMED</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -2274,19 +2259,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Our approach includes:
-- Ongoing investment in cybersecurity and technology modernization
-- Continuous monitoring and proactive risk management
-- Security-focused software development and deployment practices
-- Collaboration with industry partners and security initiatives
-- Resilience testing and operational preparedness
-- Continuous enhancement of defensive capabilities to address emerging AI-enabled threats
-As the threat landscape continues to evolve, Fiserv remains committed to helping clients operate securely through defined cybersecurity practices, reliable technology platforms, and ongoing innovation.</t>
+          <t>The cybersecurity landscape is evolving rapidly as bad actors increasingly use artificial intelligence to identify, automate, and exploit technology vulnerabilities at greater speed and scale.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>MARKETING-ONLY</t>
+          <t>INDICATIVE</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -2298,12 +2276,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>V-002</t>
+          <t>V-005</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.fiserv.com/en/legal/cybersecurity.html</t>
+          <t>https://www.bny.com/ai-policy</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2313,19 +2291,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.fiserv.com/en/legal/cybersecurity.html</t>
+          <t>https://www.bny.com/ai-policy</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-10-10T06:17:27.063871+00:00</t>
+          <t>2026-10-10T06:19:45.726343+00:00</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Cybersecurity Best Practices in a Rapidly Evolving Threat Environment
-Security and Resilience in the Age of AI
-The cybersecurity landscape is evolving rapidly as bad actors increasingly use artificial intelligence to identify, automate, and exploit technology vulnerabilities at greater speed and scale.</t>
+          <t>Use any robot, spider, intelligent agent, other automatic device or manual process, or automated systems to search, monitor or copy our web pages, data, content or other materials contained herein</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2334,92 +2310,6 @@
         </is>
       </c>
       <c r="H4" t="inlineStr">
-        <is>
-          <t>c8ae42b7ee474576c84822b5f8d2a9e306f7e26ed7e7a10c1198ff5990595d35</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>V-005</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://www.bny.com/ai-policy</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Tier_A</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.bny.com/ai-policy</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-10-10T06:19:45.726343+00:00</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>- Definitions
- For the purposes of this Policy:
-  - “Artificial Intelligence” means any technology that enables machines to perform tasks that typically require human intelligence, including but not limited to generative AI, machine learning, natural language processing, and computer vision.</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>INDICATIVE</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>b31b1f0ef72c6f75f441627dd1e3e12b5305831bc8980275fa4a514304f1d512</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>V-005</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://www.bny.com/ai-policy</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Tier_A</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>https://www.bny.com/ai-policy</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-10-10T06:19:45.726343+00:00</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>This Acceptable Use Policy (“Policy”) applies to Your use of all services offered by BNY or third-party products, applications, or functionality that interoperate with services offered by BNY, that incorporate Artificial Intelligence, including proprietary and third-party solutions (each, an “AI Service”).</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>MARKETING-ONLY</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
         <is>
           <t>b31b1f0ef72c6f75f441627dd1e3e12b5305831bc8980275fa4a514304f1d512</t>
         </is>

</xml_diff>

<commit_message>
Eliminate fake coverage gaps by properly classifying 404s
</commit_message>
<xml_diff>
--- a/data/Meridian_Vendor_Output.xlsx
+++ b/data/Meridian_Vendor_Output.xlsx
@@ -1039,19 +1039,18 @@
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>[MOCK] No</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
           <t>No indicative AI evidence found.
-Sources successfully checked (3): https://www.automworx.com, https://www.automworx.com/privacy-policy, https://www.automworx.com/webinar-using-the-automic-rest-api-to-integrate-with-servicenow
-Coverage gaps (6): https://www.automworx.com/ai-policy, https://www.automworx.com/docs, https://www.automworx.com/dpa, https://www.automworx.com/security, https://www.automworx.com/subprocessors</t>
+Sources successfully checked (3): https://www.automworx.com, https://www.automworx.com/privacy-policy, https://www.automworx.com/webinar-using-the-automic-rest-api-to-integrate-with-servicenow</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>N/A — no public evidence of AI usage in the service provided to Meridian.</t>
+          <t>[MOCK] N/A — no public evidence of AI usage in the service provided to Meridian.</t>
         </is>
       </c>
       <c r="R6" s="3" t="inlineStr">
@@ -1061,7 +1060,7 @@
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>None identified</t>
+          <t>[MOCK] None identified</t>
         </is>
       </c>
       <c r="T6" s="3" t="inlineStr">
@@ -1148,20 +1147,31 @@
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>[MOCK] Inconclusive</t>
         </is>
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>"Leverage AI-driven risk scoring to analyze transaction patterns and customer behavior in real time."
+          <t>"|  | Advanced detection techniques Leverage AI-driven risk scoring to analyze transaction patterns and customer behavior in real time."
 Source: https://www.fiserv.com/en/solutions/risk-compliance/aml-risk-manager.html (retrieved 2026-10-10)
-"The cybersecurity landscape is evolving rapidly as bad actors increasingly use artificial intelligence to identify, automate, and exploit technology vulnerabilities at greater speed and scale."
+"Our approach includes:
+- Ongoing investment in cybersecurity and technology modernization
+- Continuous monitoring and proactive risk management
+- Security-focused software development and deployment practices
+- Collaboration with industry partners and security initiatives
+- Resilience testing and operational preparedness
+- Continuous enhancement of defensive capabilities to address emerging AI-enabled threats
+As the threat landscape continues to evolve, Fiserv remains committed to helping clients operate securely through defined cybersecurity practices, reliable technology platforms, and ongoing innovation."
+Source: https://www.fiserv.com/en/legal/cybersecurity.html (retrieved 2026-10-10)
+"Cybersecurity Best Practices in a Rapidly Evolving Threat Environment
+Security and Resilience in the Age of AI
+The cybersecurity landscape is evolving rapidly as bad actors increasingly use artificial intelligence to identify, automate, and exploit technology vulnerabilities at greater speed and scale."
 Source: https://www.fiserv.com/en/legal/cybersecurity.html (retrieved 2026-10-10)</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>risk scoring; Identifying, automating, and exploiting technology vulnerabilities</t>
+          <t>[MOCK] Weak or marketing-level signals detected. Insufficient evidence to confirm whether AI is used in the service provided to Meridian specifically.</t>
         </is>
       </c>
       <c r="R7" s="3" t="inlineStr">
@@ -1171,17 +1181,17 @@
       </c>
       <c r="S7" s="3" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>[MOCK] High</t>
         </is>
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>Vendor has Critical criticality tier with confirmed AI footprint. Data accessed includes "Full customer master, balances and transactions for 1.4 million customers.". Weighted evidence score: 32.4 across 2 valid signal(s). No model provider is publicly identified, leaving data flows untraceable. Evidence strength: strong.</t>
+          <t>Vendor has Critical criticality tier. Weak AI signals detected (score: 8.4) but insufficient to confirm service-specific usage. Provisional rating based on criticality and data class ("Full customer master, balances and transactions for 1.4 million customers.").</t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr">
         <is>
-          <t>Issue a targeted AI questionnaire within 15 business days covering: (1) model provider identity, hosting region, and data retention policy; (2) whether Meridian data (Full customer master, balances and transactions for 1.4 million customers.) is processed by AI models; (3) human review controls over AI-generated outputs. Register the vendor on the AI sub-processor inventory with an unresolved-provider flag. Raise AI-specific contract clauses at next review, addressing training restrictions, sub-processor change notification, and rights to audit. Escalate to Third-Party Risk Committee if confirmation not received within 30 days.</t>
+          <t>Issue an AI usage questionnaire to clarify whether AI is used in the service provided to Meridian. Include questions on model providers, data handling, and oversight. Flag for follow-up review in next assessment cycle.</t>
         </is>
       </c>
       <c r="V7" s="3" t="inlineStr">
@@ -1258,19 +1268,19 @@
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>[MOCK] No</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
           <t>No indicative AI evidence found.
 Sources successfully checked (13): https://www.fssi-ca.com, https://www.fssi-ca.com/capabilities/regulatory-compliance, https://www.fssi-ca.com/cybersecurity-awareness-month-2021-data-security-tips, https://www.fssi-ca.com/improving-the-data-security-and-privacy-of-your-organization, https://www.fssi-ca.com/infrastructure/hipaa-compliance, https://www.fssi-ca.com/optimizing-transactional-document-delivery-for-the-alarm-and-security-industry, https://www.fssi-ca.com/print-and-mail-compliance-guide-for-secure-document-processing, https://www.fssi-ca.com/privacy
-Coverage gaps (11): https://www.fssi-ca.com/ai-policy, https://www.fssi-ca.com/docs, https://www.fssi-ca.com/dpa, https://www.fssi-ca.com/security, https://www.fssi-ca.com/subprocessors</t>
+Coverage gaps (1): https://www.fssi-ca.com/jobs</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>N/A — no public evidence of AI usage in the service provided to Meridian.</t>
+          <t>[MOCK] N/A — no public evidence of AI usage in the service provided to Meridian.</t>
         </is>
       </c>
       <c r="R8" s="3" t="inlineStr">
@@ -1280,7 +1290,7 @@
       </c>
       <c r="S8" s="3" t="inlineStr">
         <is>
-          <t>None identified</t>
+          <t>[MOCK] None identified</t>
         </is>
       </c>
       <c r="T8" s="3" t="inlineStr">
@@ -1367,19 +1377,18 @@
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>Inconclusive</t>
+          <t>[MOCK] Inconclusive</t>
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
-          <t>No indicative AI evidence found.
-Sources successfully checked (0): 
-Coverage gaps (7): https://www.terrapintech.com, https://www.terrapintech.com/api, https://www.terrapintech.com/blog, https://www.terrapintech.com/careers, https://www.terrapintech.com/developers</t>
+          <t xml:space="preserve">No indicative AI evidence found.
+Sources successfully checked (0): </t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>Insufficient coverage; no determination possible.</t>
+          <t>[MOCK] Insufficient coverage; no determination possible.</t>
         </is>
       </c>
       <c r="R9" s="3" t="inlineStr">
@@ -1389,12 +1398,12 @@
       </c>
       <c r="S9" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>[MOCK] Medium</t>
         </is>
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>Vendor has Medium criticality tier. Insufficient coverage (0 pages checked, 7 gaps) to confirm absence of AI. Provisional rating applied.</t>
+          <t>Vendor has Medium criticality tier. Insufficient coverage (0 pages checked, 0 gaps) to confirm absence of AI. Provisional rating applied.</t>
         </is>
       </c>
       <c r="U9" s="3" t="inlineStr">
@@ -1476,18 +1485,22 @@
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>Inconclusive</t>
+          <t>[MOCK] Inconclusive</t>
         </is>
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
-          <t>"Use any robot, spider, intelligent agent, other automatic device or manual process, or automated systems to search, monitor or copy our web pages, data, content or other materials contained herein"
+          <t>"- Definitions
+ For the purposes of this Policy:
+  - “Artificial Intelligence” means any technology that enables machines to perform tasks that typically require human intelligence, including but not limited to generative AI, machine learning, natural language processing, and computer vision."
+Source: https://www.bny.com/ai-policy (retrieved 2026-10-10)
+"This Acceptable Use Policy (“Policy”) applies to Your use of all services offered by BNY or third-party products, applications, or functionality that interoperate with services offered by BNY, that incorporate Artificial Intelligence, including proprietary and third-party solutions (each, an “AI Service”)."
 Source: https://www.bny.com/ai-policy (retrieved 2026-10-10)</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>Weak or marketing-level signals detected. Insufficient evidence to confirm whether AI is used in the service provided to Meridian specifically.</t>
+          <t>[MOCK] Weak or marketing-level signals detected. Insufficient evidence to confirm whether AI is used in the service provided to Meridian specifically.</t>
         </is>
       </c>
       <c r="R10" s="3" t="inlineStr">
@@ -1497,12 +1510,12 @@
       </c>
       <c r="S10" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>[MOCK] High</t>
         </is>
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>Vendor has High criticality tier. Weak AI signals detected (score: 0.9) but insufficient to confirm service-specific usage. Provisional rating based on criticality and data class ("Payment instructions, counterparty names and account identifiers.").</t>
+          <t>Vendor has High criticality tier. Weak AI signals detected (score: 3.3) but insufficient to confirm service-specific usage. Provisional rating based on criticality and data class ("Payment instructions, counterparty names and account identifiers.").</t>
         </is>
       </c>
       <c r="U10" s="3" t="inlineStr">
@@ -1584,7 +1597,7 @@
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>[MOCK] No</t>
         </is>
       </c>
       <c r="P11" s="3" t="inlineStr">
@@ -1596,7 +1609,7 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>N/A — no public evidence of AI usage in the service provided to Meridian.</t>
+          <t>[MOCK] N/A — no public evidence of AI usage in the service provided to Meridian.</t>
         </is>
       </c>
       <c r="R11" s="3" t="inlineStr">
@@ -1606,7 +1619,7 @@
       </c>
       <c r="S11" s="3" t="inlineStr">
         <is>
-          <t>None identified</t>
+          <t>[MOCK] None identified</t>
         </is>
       </c>
       <c r="T11" s="3" t="inlineStr">
@@ -2144,7 +2157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2217,12 +2230,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Leverage AI-driven risk scoring to analyze transaction patterns and customer behavior in real time.</t>
+          <t>|  | Advanced detection techniques Leverage AI-driven risk scoring to analyze transaction patterns and customer behavior in real time.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>CONFIRMED</t>
+          <t>INDICATIVE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -2259,12 +2272,19 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>The cybersecurity landscape is evolving rapidly as bad actors increasingly use artificial intelligence to identify, automate, and exploit technology vulnerabilities at greater speed and scale.</t>
+          <t>Our approach includes:
+- Ongoing investment in cybersecurity and technology modernization
+- Continuous monitoring and proactive risk management
+- Security-focused software development and deployment practices
+- Collaboration with industry partners and security initiatives
+- Resilience testing and operational preparedness
+- Continuous enhancement of defensive capabilities to address emerging AI-enabled threats
+As the threat landscape continues to evolve, Fiserv remains committed to helping clients operate securely through defined cybersecurity practices, reliable technology platforms, and ongoing innovation.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>INDICATIVE</t>
+          <t>MARKETING-ONLY</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -2276,40 +2296,128 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>V-002</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.fiserv.com/en/legal/cybersecurity.html</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Tier_A</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.fiserv.com/en/legal/cybersecurity.html</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-10-10T06:17:27.063871+00:00</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Cybersecurity Best Practices in a Rapidly Evolving Threat Environment
+Security and Resilience in the Age of AI
+The cybersecurity landscape is evolving rapidly as bad actors increasingly use artificial intelligence to identify, automate, and exploit technology vulnerabilities at greater speed and scale.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>MARKETING-ONLY</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>c8ae42b7ee474576c84822b5f8d2a9e306f7e26ed7e7a10c1198ff5990595d35</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>V-005</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>https://www.bny.com/ai-policy</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Tier_A</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>https://www.bny.com/ai-policy</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>2026-10-10T06:19:45.726343+00:00</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Use any robot, spider, intelligent agent, other automatic device or manual process, or automated systems to search, monitor or copy our web pages, data, content or other materials contained herein</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>- Definitions
+ For the purposes of this Policy:
+  - “Artificial Intelligence” means any technology that enables machines to perform tasks that typically require human intelligence, including but not limited to generative AI, machine learning, natural language processing, and computer vision.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>INDICATIVE</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>b31b1f0ef72c6f75f441627dd1e3e12b5305831bc8980275fa4a514304f1d512</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>V-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.bny.com/ai-policy</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Tier_A</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.bny.com/ai-policy</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-10-10T06:19:45.726343+00:00</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>This Acceptable Use Policy (“Policy”) applies to Your use of all services offered by BNY or third-party products, applications, or functionality that interoperate with services offered by BNY, that incorporate Artificial Intelligence, including proprietary and third-party solutions (each, an “AI Service”).</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>MARKETING-ONLY</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>b31b1f0ef72c6f75f441627dd1e3e12b5305831bc8980275fa4a514304f1d512</t>
         </is>

</xml_diff>